<commit_message>
separate Symbol availability from schematic names in CE handoff
</commit_message>
<xml_diff>
--- a/public/material-ce-reference.xlsx
+++ b/public/material-ce-reference.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分工與欄位說明" sheetId="1" r:id="Rfa1685f3c5b34075"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CE交付範例" sheetId="2" r:id="R40c4de49d6c94f5d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分工與欄位說明" sheetId="1" r:id="R4d968862b34f4961"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CE交付範例" sheetId="2" r:id="Rb9288c9fc20e4ce5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -722,12 +722,16 @@
       <x:c r="D16" s="23"/>
       <x:c r="E16" s="23"/>
     </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="3"/>
-      <x:c r="B17" s="3"/>
-      <x:c r="C17" s="3"/>
-      <x:c r="D17" s="3"/>
-      <x:c r="E17" s="3"/>
+    <x:row r="17" ht="58" customHeight="1">
+      <x:c r="A17" s="23" t="str">
+        <x:v>規則 6</x:v>
+      </x:c>
+      <x:c r="B17" s="23"/>
+      <x:c r="C17" s="22" t="str">
+        <x:v>Symbol 填該料號是否已建置 Symbol：有／無／待確認。已有 Part、明確無 Symbol 時只補 Symbol；空白或 C 等未定義代碼保留原值，先待確認。Schematic_Part 另存符號名稱。</x:v>
+      </x:c>
+      <x:c r="D17" s="23"/>
+      <x:c r="E17" s="23"/>
     </x:row>
     <x:row r="18" ht="27" customHeight="1">
       <x:c r="A18" s="9" t="str">
@@ -1064,88 +1068,105 @@
         <x:v>000-DEMO-001</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="34" customHeight="1">
+    <x:row r="41" ht="52" customHeight="1">
       <x:c r="A41" s="27" t="str">
-        <x:v>Part Name</x:v>
+        <x:v>Symbol</x:v>
       </x:c>
       <x:c r="B41" s="27" t="str">
-        <x:v>CE 從公司系統帶出</x:v>
+        <x:v>CE 查核後填寫</x:v>
       </x:c>
       <x:c r="C41" s="28" t="str">
-        <x:v>來源有公司料名就保留；無資料可留白。</x:v>
+        <x:v>填該料號有沒有已建置 Symbol：有／無／待確認。已有 Part 且填無時只需補 Symbol；原始 C 等代碼保留，未定義前不判有無。</x:v>
       </x:c>
       <x:c r="D41" s="28" t="str">
-        <x:v>內部料名</x:v>
+        <x:v>Symbol 建置狀態／缺件提示</x:v>
       </x:c>
       <x:c r="E41" s="32" t="str">
-        <x:v>示範電容</x:v>
+        <x:v>有／無／待確認</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="34" customHeight="1">
       <x:c r="A42" s="27" t="str">
-        <x:v>Part Spec</x:v>
+        <x:v>Part Name</x:v>
       </x:c>
       <x:c r="B42" s="27" t="str">
-        <x:v>RD 原始／CE 保留</x:v>
+        <x:v>CE 從公司系統帶出</x:v>
       </x:c>
       <x:c r="C42" s="28" t="str">
-        <x:v>保留原規格；同組資料維持一致，差異交 RD 確認。</x:v>
+        <x:v>來源有公司料名就保留；無資料可留白。</x:v>
       </x:c>
       <x:c r="D42" s="28" t="str">
-        <x:v>規格</x:v>
+        <x:v>內部料名</x:v>
       </x:c>
       <x:c r="E42" s="32" t="str">
-        <x:v>0.1uF / 16V / X7R</x:v>
+        <x:v>示範電容</x:v>
       </x:c>
     </x:row>
     <x:row r="43" ht="34" customHeight="1">
       <x:c r="A43" s="27" t="str">
-        <x:v>Schematic_Part</x:v>
+        <x:v>Part Spec</x:v>
       </x:c>
       <x:c r="B43" s="27" t="str">
         <x:v>RD 原始／CE 保留</x:v>
       </x:c>
       <x:c r="C43" s="28" t="str">
-        <x:v>原 BOM 有原理圖符號就保留；無資料可留白，不要求 CE 新建符號。</x:v>
+        <x:v>保留原規格；同組資料維持一致，差異交 RD 確認。</x:v>
       </x:c>
       <x:c r="D43" s="28" t="str">
-        <x:v>Symbol</x:v>
+        <x:v>規格</x:v>
       </x:c>
       <x:c r="E43" s="32" t="str">
-        <x:v>CAP</x:v>
+        <x:v>0.1uF / 16V / X7R</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="34" customHeight="1">
       <x:c r="A44" s="27" t="str">
+        <x:v>Schematic_Part</x:v>
+      </x:c>
+      <x:c r="B44" s="27" t="str">
+        <x:v>原 BOM／CE 保留</x:v>
+      </x:c>
+      <x:c r="C44" s="28" t="str">
+        <x:v>原 BOM 的符號名稱，例如 CAP；這欄不代表 Symbol 是否已建置，有無狀態請填 Symbol 欄。</x:v>
+      </x:c>
+      <x:c r="D44" s="28" t="str">
+        <x:v>原理圖符號名稱</x:v>
+      </x:c>
+      <x:c r="E44" s="32" t="str">
+        <x:v>CAP</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="34" customHeight="1">
+      <x:c r="A45" s="27" t="str">
         <x:v>PCB_Footprint</x:v>
       </x:c>
-      <x:c r="B44" s="27" t="str">
+      <x:c r="B45" s="27" t="str">
         <x:v>RD 原始／CE 保留</x:v>
       </x:c>
-      <x:c r="C44" s="28" t="str">
+      <x:c r="C45" s="28" t="str">
         <x:v>原 BOM 有封裝就保留；無資料可留白，不要求 CE 新建封裝。</x:v>
       </x:c>
-      <x:c r="D44" s="28" t="str">
+      <x:c r="D45" s="28" t="str">
         <x:v>Footprint</x:v>
       </x:c>
-      <x:c r="E44" s="32" t="str">
+      <x:c r="E45" s="32" t="str">
         <x:v>C_0402</x:v>
       </x:c>
     </x:row>
-    <x:row r="45" ht="34" customHeight="1">
-      <x:c r="A45" s="29" t="str">
+    <x:row r="46" ht="34" customHeight="1">
+      <x:c r="A46" s="29" t="str">
         <x:v>零件狀態</x:v>
       </x:c>
-      <x:c r="B45" s="29" t="str">
+      <x:c r="B46" s="29" t="str">
         <x:v>CE 補欄／帶出原文</x:v>
       </x:c>
-      <x:c r="C45" s="30" t="str">
+      <x:c r="C46" s="30" t="str">
         <x:v>本次交付必須補在最右側。填公司新設計使用限制原文；不明填待確認，供 RD 後續確認與參考。</x:v>
       </x:c>
-      <x:c r="D45" s="30" t="str">
+      <x:c r="D46" s="30" t="str">
         <x:v>零件狀態（獨立顯示）</x:v>
       </x:c>
-      <x:c r="E45" s="33" t="str">
+      <x:c r="E46" s="33" t="str">
         <x:v>新設計產品不建議使用－ODM 不建議用料</x:v>
       </x:c>
     </x:row>
@@ -1175,11 +1196,12 @@
     <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="30" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="25" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="25" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="30" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="25" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="26" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="25" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="30" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="25" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="45" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="25" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="45" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1204,6 +1226,7 @@
       <x:c r="Q1" s="6"/>
       <x:c r="R1" s="6"/>
       <x:c r="S1" s="6"/>
+      <x:c r="T1" s="6"/>
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="34" t="str">
@@ -1227,6 +1250,7 @@
       <x:c r="Q2" s="3"/>
       <x:c r="R2" s="3"/>
       <x:c r="S2" s="3"/>
+      <x:c r="T2" s="3"/>
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="37" t="str">
@@ -1281,21 +1305,24 @@
         <x:v>CE 從公司系統帶出</x:v>
       </x:c>
       <x:c r="O3" s="37" t="str">
+        <x:v>CE 查核後填寫</x:v>
+      </x:c>
+      <x:c r="P3" s="37" t="str">
         <x:v>CE 從公司系統帶出</x:v>
-      </x:c>
-      <x:c r="P3" s="37" t="str">
-        <x:v>RD 原始
-CE 保留</x:v>
       </x:c>
       <x:c r="Q3" s="37" t="str">
         <x:v>RD 原始
 CE 保留</x:v>
       </x:c>
       <x:c r="R3" s="37" t="str">
+        <x:v>原 BOM
+CE 保留</x:v>
+      </x:c>
+      <x:c r="S3" s="37" t="str">
         <x:v>RD 原始
 CE 保留</x:v>
       </x:c>
-      <x:c r="S3" s="38" t="str">
+      <x:c r="T3" s="38" t="str">
         <x:v>CE 補欄
 帶出原文</x:v>
       </x:c>
@@ -1344,18 +1371,21 @@
         <x:v>Part Number</x:v>
       </x:c>
       <x:c r="O4" s="19" t="str">
+        <x:v>Symbol</x:v>
+      </x:c>
+      <x:c r="P4" s="19" t="str">
         <x:v>Part Name</x:v>
       </x:c>
-      <x:c r="P4" s="19" t="str">
+      <x:c r="Q4" s="19" t="str">
         <x:v>Part Spec</x:v>
       </x:c>
-      <x:c r="Q4" s="19" t="str">
+      <x:c r="R4" s="19" t="str">
         <x:v>Schematic_Part</x:v>
       </x:c>
-      <x:c r="R4" s="19" t="str">
+      <x:c r="S4" s="19" t="str">
         <x:v>PCB_Footprint</x:v>
       </x:c>
-      <x:c r="S4" s="20" t="str">
+      <x:c r="T4" s="20" t="str">
         <x:v>零件狀態</x:v>
       </x:c>
     </x:row>
@@ -1399,18 +1429,21 @@
         <x:v>000-DEMO-001</x:v>
       </x:c>
       <x:c r="O5" s="45" t="str">
+        <x:v>無</x:v>
+      </x:c>
+      <x:c r="P5" s="45" t="str">
         <x:v>示範電容</x:v>
       </x:c>
-      <x:c r="P5" s="45" t="str">
+      <x:c r="Q5" s="45" t="str">
         <x:v>0.1uF / 16V / X7R</x:v>
       </x:c>
-      <x:c r="Q5" s="45" t="str">
+      <x:c r="R5" s="45" t="str">
         <x:v>CAP</x:v>
       </x:c>
-      <x:c r="R5" s="45" t="str">
+      <x:c r="S5" s="45" t="str">
         <x:v>C_0402</x:v>
       </x:c>
-      <x:c r="S5" s="45" t="str">
+      <x:c r="T5" s="45" t="str">
         <x:v>待確認</x:v>
       </x:c>
     </x:row>
@@ -1454,18 +1487,21 @@
         <x:v>000-DEMO-ALT</x:v>
       </x:c>
       <x:c r="O6" s="46" t="str">
+        <x:v>C</x:v>
+      </x:c>
+      <x:c r="P6" s="46" t="str">
         <x:v>示範替代電容</x:v>
       </x:c>
-      <x:c r="P6" s="46" t="str">
+      <x:c r="Q6" s="46" t="str">
         <x:v>0.1uF / 16V / X7R</x:v>
       </x:c>
-      <x:c r="Q6" s="46" t="str">
+      <x:c r="R6" s="46" t="str">
         <x:v>CAP</x:v>
       </x:c>
-      <x:c r="R6" s="46" t="str">
+      <x:c r="S6" s="46" t="str">
         <x:v>C_0402</x:v>
       </x:c>
-      <x:c r="S6" s="46" t="str">
+      <x:c r="T6" s="46" t="str">
         <x:v>新設計產品不建議使用－ODM 不建議用料</x:v>
       </x:c>
     </x:row>
@@ -1507,18 +1543,21 @@
         <x:v>000-DEMO-EOL</x:v>
       </x:c>
       <x:c r="O7" s="46" t="str">
+        <x:v>有</x:v>
+      </x:c>
+      <x:c r="P7" s="46" t="str">
         <x:v>示範電源 IC</x:v>
       </x:c>
-      <x:c r="P7" s="46" t="str">
+      <x:c r="Q7" s="46" t="str">
         <x:v>示範規格</x:v>
       </x:c>
-      <x:c r="Q7" s="46" t="str">
+      <x:c r="R7" s="46" t="str">
         <x:v>POWER_IC</x:v>
       </x:c>
-      <x:c r="R7" s="46" t="str">
+      <x:c r="S7" s="46" t="str">
         <x:v>QFN_DEMO</x:v>
       </x:c>
-      <x:c r="S7" s="46" t="str">
+      <x:c r="T7" s="46" t="str">
         <x:v>新設計產品不建議使用－EOL</x:v>
       </x:c>
     </x:row>
@@ -1555,17 +1594,20 @@
         <x:v>查無公司料號；請 RD 確認後續處理</x:v>
       </x:c>
       <x:c r="N8" s="47" t="str"/>
-      <x:c r="O8" s="47" t="str"/>
-      <x:c r="P8" s="47" t="str">
+      <x:c r="O8" s="47" t="str">
+        <x:v>無</x:v>
+      </x:c>
+      <x:c r="P8" s="47" t="str"/>
+      <x:c r="Q8" s="47" t="str">
         <x:v>示範規格</x:v>
       </x:c>
-      <x:c r="Q8" s="47" t="str">
+      <x:c r="R8" s="47" t="str">
         <x:v>CONN</x:v>
       </x:c>
-      <x:c r="R8" s="47" t="str">
+      <x:c r="S8" s="47" t="str">
         <x:v>CONN_DEMO</x:v>
       </x:c>
-      <x:c r="S8" s="47" t="str">
+      <x:c r="T8" s="47" t="str">
         <x:v>待確認</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
align CE handoff with virtual and physical part numbers
</commit_message>
<xml_diff>
--- a/public/material-ce-reference.xlsx
+++ b/public/material-ce-reference.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分工與欄位說明" sheetId="1" r:id="R4d968862b34f4961"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CE交付範例" sheetId="2" r:id="Rb9288c9fc20e4ce5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分工與欄位說明" sheetId="1" r:id="R0c4ec5f9217b4f2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CE交付範例" sheetId="2" r:id="Ref6b92ebbffa442d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -633,7 +633,7 @@
         <x:v>可檢查的料號總表與追蹤紀錄</x:v>
       </x:c>
       <x:c r="C8" s="22" t="str">
-        <x:v>自動讀取欄位、整理主料與替代料、對應 TX、呈現料號與風險；保留原文，不代替公司系統核准料號，也不替 RD 決定能否採用。</x:v>
+        <x:v>自動讀取欄位、整理同一虛擬料號下的實體料，呈現料號與風險；保留原文，不代替公司系統核准料號，也不替 RD 決定能否採用。</x:v>
       </x:c>
       <x:c r="D8" s="3"/>
       <x:c r="E8" s="3"/>
@@ -678,7 +678,7 @@
       <x:c r="D12" s="23"/>
       <x:c r="E12" s="23"/>
     </x:row>
-    <x:row r="13" ht="44" customHeight="1">
+    <x:row r="13" ht="58" customHeight="1">
       <x:c r="A13" s="23" t="str">
         <x:v>規則 2</x:v>
       </x:c>
@@ -695,7 +695,7 @@
       </x:c>
       <x:c r="B14" s="23"/>
       <x:c r="C14" s="22" t="str">
-        <x:v>零件狀態放在 BOM 最右側，由 CE 帶出公司原文；未確認時填待確認，不得自行改填 Approved 或可用。查無公司料號時，Part Number 保持空白。</x:v>
+        <x:v>料號只有兩種：實體料號對應單一廠商的單一廠商料號；虛擬料號是可共用實體料的群組。同一虛擬料號下的實體料各列一行；查無實體料號時留白，不用虛擬料號代填。</x:v>
       </x:c>
       <x:c r="D14" s="23"/>
       <x:c r="E14" s="23"/>
@@ -728,7 +728,7 @@
       </x:c>
       <x:c r="B17" s="23"/>
       <x:c r="C17" s="22" t="str">
-        <x:v>Symbol 填該料號是否已建置 Symbol：有／無／待確認。已有 Part、明確無 Symbol 時只補 Symbol；空白或 C 等未定義代碼保留原值，先待確認。Schematic_Part 另存符號名稱。</x:v>
+        <x:v>Symbol 填該實體料是否已建置 Symbol：有／無／待確認。已有實體料號、明確無 Symbol 時只補 Symbol；空白或 C 等未定義代碼保留原值，先待確認。Schematic_Part 另存符號名稱。</x:v>
       </x:c>
       <x:c r="D17" s="23"/>
       <x:c r="E17" s="23"/>
@@ -759,7 +759,7 @@
       </x:c>
       <x:c r="B20" s="23"/>
       <x:c r="C20" s="22" t="str">
-        <x:v>CE 利用公司現有系統核對並帶出公司料號、供應狀態等資料，在最右側補上零件狀態；未知處明確填待確認。</x:v>
+        <x:v>CE 利用公司現有系統核對並帶出虛擬料號、實體料號與供應狀態，在最右側補上零件狀態；未知處明確填待確認。</x:v>
       </x:c>
       <x:c r="D20" s="23"/>
       <x:c r="E20" s="23"/>
@@ -770,7 +770,7 @@
       </x:c>
       <x:c r="B21" s="23"/>
       <x:c r="C21" s="22" t="str">
-        <x:v>CE 依空白範本的固定表頭交付 Excel；一列一個廠商料，同組替代料相鄰排列，保留 Ref_tmp／Ref Des。</x:v>
+        <x:v>CE 依空白範本的固定表頭交付 Excel；每列為單一廠商的一個實體料，同一虛擬料下的實體料分列填寫，保留 Ref Des。</x:v>
       </x:c>
       <x:c r="D21" s="23"/>
       <x:c r="E21" s="23"/>
@@ -781,7 +781,7 @@
       </x:c>
       <x:c r="B22" s="23"/>
       <x:c r="C22" s="22" t="str">
-        <x:v>RD 使用上傳 BOM 匯入，核對群組數、位號、MPN、公司料號、供應狀態與零件狀態。工具只整理與提示，不自動核准。</x:v>
+        <x:v>RD 使用上傳 BOM 匯入，核對位號、MPN、虛擬料號、實體料號、供應狀態與零件狀態。工具只整理與提示，不自動核准。</x:v>
       </x:c>
       <x:c r="D22" s="23"/>
       <x:c r="E22" s="23"/>
@@ -900,13 +900,13 @@
     </x:row>
     <x:row r="31" ht="34" customHeight="1">
       <x:c r="A31" s="27" t="str">
-        <x:v>Manufacturer Part Number(1)</x:v>
+        <x:v>Manufacturer Part Number</x:v>
       </x:c>
       <x:c r="B31" s="27" t="str">
         <x:v>RD 提供／CE 核對</x:v>
       </x:c>
       <x:c r="C31" s="28" t="str">
-        <x:v>每列一個廠商料號；依原 BOM 與公司資料核對，不自行換成未確認替代料。</x:v>
+        <x:v>每列只填一個廠商料號，搭配該列廠商及實體料號；同一虛擬料下的其他實體料另列。</x:v>
       </x:c>
       <x:c r="D31" s="28" t="str">
         <x:v>MPN</x:v>
@@ -917,256 +917,171 @@
     </x:row>
     <x:row r="32" ht="34" customHeight="1">
       <x:c r="A32" s="27" t="str">
-        <x:v>Manufacturer Part Number(2)</x:v>
+        <x:v>Manufacturer</x:v>
       </x:c>
       <x:c r="B32" s="27" t="str">
-        <x:v>CE 保留舊格式</x:v>
+        <x:v>CE 核對／帶出</x:v>
       </x:c>
       <x:c r="C32" s="28" t="str">
-        <x:v>舊格式相容欄，可留白；新交付的其他候選料請各自另列。</x:v>
+        <x:v>填該列 MPN 對應的廠商，不把不同廠商合在同一列。</x:v>
       </x:c>
       <x:c r="D32" s="28" t="str">
-        <x:v>第二 MPN（相容欄）</x:v>
+        <x:v>廠商</x:v>
       </x:c>
       <x:c r="E32" s="32" t="str">
-        <x:v>留白</x:v>
+        <x:v>示範廠商 A</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="34" customHeight="1">
       <x:c r="A33" s="27" t="str">
-        <x:v>Manufacturer</x:v>
+        <x:v>Sourcing Status</x:v>
       </x:c>
       <x:c r="B33" s="27" t="str">
-        <x:v>CE 核對／帶出</x:v>
+        <x:v>CE 從來源帶出</x:v>
       </x:c>
       <x:c r="C33" s="28" t="str">
-        <x:v>填該列 MPN 對應的廠商，不把不同廠商合在同一列。</x:v>
+        <x:v>保留公司／原廠供應與核准狀態原文，例如 Approved、Active、NRND、Obsolete；不得用它取代右側零件狀態。</x:v>
       </x:c>
       <x:c r="D33" s="28" t="str">
-        <x:v>廠商</x:v>
+        <x:v>供應／核准狀態</x:v>
       </x:c>
       <x:c r="E33" s="32" t="str">
-        <x:v>示範廠商 A</x:v>
+        <x:v>Approved</x:v>
       </x:c>
     </x:row>
     <x:row r="34" ht="34" customHeight="1">
       <x:c r="A34" s="27" t="str">
-        <x:v>Sourcing Status</x:v>
+        <x:v>虛擬料號</x:v>
       </x:c>
       <x:c r="B34" s="27" t="str">
-        <x:v>CE 從來源帶出</x:v>
+        <x:v>CE 從公司系統帶出</x:v>
       </x:c>
       <x:c r="C34" s="28" t="str">
-        <x:v>保留公司／原廠供應與核准狀態原文，例如 Approved、Active、NRND、Obsolete；不得用它取代右側零件狀態。</x:v>
+        <x:v>填可共用實體料的虛擬料號；同一群組的實體料重複填相同虛擬料號。來源無值留白，不自行編號。</x:v>
       </x:c>
       <x:c r="D34" s="28" t="str">
-        <x:v>供應／核准狀態</x:v>
+        <x:v>虛擬料號</x:v>
       </x:c>
       <x:c r="E34" s="32" t="str">
-        <x:v>Approved</x:v>
+        <x:v>DEMO-VIRTUAL-001</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="34" customHeight="1">
       <x:c r="A35" s="27" t="str">
-        <x:v>Virtual PN</x:v>
+        <x:v>實體料號</x:v>
       </x:c>
       <x:c r="B35" s="27" t="str">
-        <x:v>CE 從來源帶出</x:v>
+        <x:v>CE 從公司系統帶出</x:v>
       </x:c>
       <x:c r="C35" s="28" t="str">
-        <x:v>來源有值才帶出；無值留白，不要自編 TX。</x:v>
+        <x:v>填已申請的實體料號，每個料號對應單一廠商、單一 MPN，並保留前導零。查無時留白，不以虛擬料號或 MPN 代填。</x:v>
       </x:c>
       <x:c r="D35" s="28" t="str">
-        <x:v>TX（第一優先）</x:v>
+        <x:v>實體料號</x:v>
       </x:c>
       <x:c r="E35" s="32" t="str">
-        <x:v>DEMO-TX-001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36" ht="34" customHeight="1">
+        <x:v>000-DEMO-001</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="52" customHeight="1">
       <x:c r="A36" s="27" t="str">
-        <x:v>PEGA P/N</x:v>
+        <x:v>Symbol</x:v>
       </x:c>
       <x:c r="B36" s="27" t="str">
-        <x:v>CE 從來源帶出</x:v>
+        <x:v>CE 查核後填寫</x:v>
       </x:c>
       <x:c r="C36" s="28" t="str">
-        <x:v>來源有值才帶出；Virtual PN 空白時才作為 TX 後備值，無值留白。</x:v>
+        <x:v>填該實體料有沒有已建置 Symbol：有／無／待確認。已有實體料號且填無時只需補 Symbol；原始 C 等代碼保留，未定義前不判有無。</x:v>
       </x:c>
       <x:c r="D36" s="28" t="str">
-        <x:v>TX（第二優先）</x:v>
+        <x:v>Symbol 建置狀態／缺件提示</x:v>
       </x:c>
       <x:c r="E36" s="32" t="str">
-        <x:v>DEMO-PEGA-001</x:v>
+        <x:v>有／無／待確認</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="34" customHeight="1">
       <x:c r="A37" s="27" t="str">
-        <x:v>Ref_tmp</x:v>
+        <x:v>Part Name</x:v>
       </x:c>
       <x:c r="B37" s="27" t="str">
-        <x:v>原始分組／CE 保留</x:v>
+        <x:v>CE 從公司系統帶出</x:v>
       </x:c>
       <x:c r="C37" s="28" t="str">
-        <x:v>可留白由工具依 Ref Des 分組；本範本若填寫，使用與 Ref Des 相同的完整位號集合，同組替代料相鄰排列。</x:v>
+        <x:v>來源有公司料名就保留；無資料可留白。</x:v>
       </x:c>
       <x:c r="D37" s="28" t="str">
-        <x:v>Ref Group</x:v>
+        <x:v>內部料名</x:v>
       </x:c>
       <x:c r="E37" s="32" t="str">
-        <x:v>C101, C102</x:v>
+        <x:v>示範電容</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="34" customHeight="1">
       <x:c r="A38" s="27" t="str">
-        <x:v>LV</x:v>
+        <x:v>Part Spec</x:v>
       </x:c>
       <x:c r="B38" s="27" t="str">
-        <x:v>來源資料／CE 保留</x:v>
+        <x:v>RD 原始／CE 保留</x:v>
       </x:c>
       <x:c r="C38" s="28" t="str">
-        <x:v>來源有版次就保留，不另造版本。</x:v>
+        <x:v>保留原規格；同組資料維持一致，差異交 RD 確認。</x:v>
       </x:c>
       <x:c r="D38" s="28" t="str">
-        <x:v>版次</x:v>
+        <x:v>規格</x:v>
       </x:c>
       <x:c r="E38" s="32" t="str">
-        <x:v>A</x:v>
+        <x:v>0.1uF / 16V / X7R</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="34" customHeight="1">
       <x:c r="A39" s="27" t="str">
-        <x:v>CIS/Remark</x:v>
+        <x:v>Schematic_Part</x:v>
       </x:c>
       <x:c r="B39" s="27" t="str">
-        <x:v>來源參考／CE 保留</x:v>
+        <x:v>原 BOM／CE 保留</x:v>
       </x:c>
       <x:c r="C39" s="28" t="str">
-        <x:v>只供原 Excel 參考；網站不匯入此欄，也不把它當成 RD 追蹤說明。</x:v>
+        <x:v>原 BOM 的符號名稱，例如 CAP；這欄不代表 Symbol 是否已建置，有無狀態請填 Symbol 欄。</x:v>
       </x:c>
       <x:c r="D39" s="28" t="str">
-        <x:v>不匯入</x:v>
+        <x:v>原理圖符號名稱</x:v>
       </x:c>
       <x:c r="E39" s="32" t="str">
-        <x:v>來源備註（選填）</x:v>
+        <x:v>CAP</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="34" customHeight="1">
       <x:c r="A40" s="27" t="str">
-        <x:v>Part Number</x:v>
+        <x:v>PCB_Footprint</x:v>
       </x:c>
       <x:c r="B40" s="27" t="str">
-        <x:v>CE 從公司系統帶出</x:v>
+        <x:v>RD 原始／CE 保留</x:v>
       </x:c>
       <x:c r="C40" s="28" t="str">
-        <x:v>填公司正式料號並保留前導零；查無時留白，於零件狀態填待確認，不把廠商 MPN／TX 填進這欄。</x:v>
+        <x:v>原 BOM 有封裝就保留；無資料可留白，不要求 CE 新建封裝。</x:v>
       </x:c>
       <x:c r="D40" s="28" t="str">
-        <x:v>內部料號</x:v>
+        <x:v>Footprint</x:v>
       </x:c>
       <x:c r="E40" s="32" t="str">
-        <x:v>000-DEMO-001</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="41" ht="52" customHeight="1">
-      <x:c r="A41" s="27" t="str">
-        <x:v>Symbol</x:v>
-      </x:c>
-      <x:c r="B41" s="27" t="str">
-        <x:v>CE 查核後填寫</x:v>
-      </x:c>
-      <x:c r="C41" s="28" t="str">
-        <x:v>填該料號有沒有已建置 Symbol：有／無／待確認。已有 Part 且填無時只需補 Symbol；原始 C 等代碼保留，未定義前不判有無。</x:v>
-      </x:c>
-      <x:c r="D41" s="28" t="str">
-        <x:v>Symbol 建置狀態／缺件提示</x:v>
-      </x:c>
-      <x:c r="E41" s="32" t="str">
-        <x:v>有／無／待確認</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="34" customHeight="1">
-      <x:c r="A42" s="27" t="str">
-        <x:v>Part Name</x:v>
-      </x:c>
-      <x:c r="B42" s="27" t="str">
-        <x:v>CE 從公司系統帶出</x:v>
-      </x:c>
-      <x:c r="C42" s="28" t="str">
-        <x:v>來源有公司料名就保留；無資料可留白。</x:v>
-      </x:c>
-      <x:c r="D42" s="28" t="str">
-        <x:v>內部料名</x:v>
-      </x:c>
-      <x:c r="E42" s="32" t="str">
-        <x:v>示範電容</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="43" ht="34" customHeight="1">
-      <x:c r="A43" s="27" t="str">
-        <x:v>Part Spec</x:v>
-      </x:c>
-      <x:c r="B43" s="27" t="str">
-        <x:v>RD 原始／CE 保留</x:v>
-      </x:c>
-      <x:c r="C43" s="28" t="str">
-        <x:v>保留原規格；同組資料維持一致，差異交 RD 確認。</x:v>
-      </x:c>
-      <x:c r="D43" s="28" t="str">
-        <x:v>規格</x:v>
-      </x:c>
-      <x:c r="E43" s="32" t="str">
-        <x:v>0.1uF / 16V / X7R</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44" ht="34" customHeight="1">
-      <x:c r="A44" s="27" t="str">
-        <x:v>Schematic_Part</x:v>
-      </x:c>
-      <x:c r="B44" s="27" t="str">
-        <x:v>原 BOM／CE 保留</x:v>
-      </x:c>
-      <x:c r="C44" s="28" t="str">
-        <x:v>原 BOM 的符號名稱，例如 CAP；這欄不代表 Symbol 是否已建置，有無狀態請填 Symbol 欄。</x:v>
-      </x:c>
-      <x:c r="D44" s="28" t="str">
-        <x:v>原理圖符號名稱</x:v>
-      </x:c>
-      <x:c r="E44" s="32" t="str">
-        <x:v>CAP</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45" ht="34" customHeight="1">
-      <x:c r="A45" s="27" t="str">
-        <x:v>PCB_Footprint</x:v>
-      </x:c>
-      <x:c r="B45" s="27" t="str">
-        <x:v>RD 原始／CE 保留</x:v>
-      </x:c>
-      <x:c r="C45" s="28" t="str">
-        <x:v>原 BOM 有封裝就保留；無資料可留白，不要求 CE 新建封裝。</x:v>
-      </x:c>
-      <x:c r="D45" s="28" t="str">
-        <x:v>Footprint</x:v>
-      </x:c>
-      <x:c r="E45" s="32" t="str">
         <x:v>C_0402</x:v>
       </x:c>
     </x:row>
-    <x:row r="46" ht="34" customHeight="1">
-      <x:c r="A46" s="29" t="str">
+    <x:row r="41" ht="34" customHeight="1">
+      <x:c r="A41" s="29" t="str">
         <x:v>零件狀態</x:v>
       </x:c>
-      <x:c r="B46" s="29" t="str">
+      <x:c r="B41" s="29" t="str">
         <x:v>CE 補欄／帶出原文</x:v>
       </x:c>
-      <x:c r="C46" s="30" t="str">
+      <x:c r="C41" s="30" t="str">
         <x:v>本次交付必須補在最右側。填公司新設計使用限制原文；不明填待確認，供 RD 後續確認與參考。</x:v>
       </x:c>
-      <x:c r="D46" s="30" t="str">
+      <x:c r="D41" s="30" t="str">
         <x:v>零件狀態（獨立顯示）</x:v>
       </x:c>
-      <x:c r="E46" s="33" t="str">
+      <x:c r="E41" s="33" t="str">
         <x:v>新設計產品不建議使用－ODM 不建議用料</x:v>
       </x:c>
     </x:row>
@@ -1187,21 +1102,16 @@
     <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="24" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="32" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="32" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="24" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="25" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="25" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="23" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="23" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="28" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="26" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="25" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="12" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="30" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="30" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="25" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="25" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="26" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="25" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="30" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="25" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="25" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="45" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="45" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1222,11 +1132,6 @@
       <x:c r="M1" s="6"/>
       <x:c r="N1" s="6"/>
       <x:c r="O1" s="6"/>
-      <x:c r="P1" s="6"/>
-      <x:c r="Q1" s="6"/>
-      <x:c r="R1" s="6"/>
-      <x:c r="S1" s="6"/>
-      <x:c r="T1" s="6"/>
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="34" t="str">
@@ -1246,11 +1151,6 @@
       <x:c r="M2" s="3"/>
       <x:c r="N2" s="3"/>
       <x:c r="O2" s="3"/>
-      <x:c r="P2" s="3"/>
-      <x:c r="Q2" s="3"/>
-      <x:c r="R2" s="3"/>
-      <x:c r="S2" s="3"/>
-      <x:c r="T2" s="3"/>
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="37" t="str">
@@ -1274,55 +1174,37 @@
 CE 核對</x:v>
       </x:c>
       <x:c r="F3" s="37" t="str">
-        <x:v>CE 保留舊格式</x:v>
-      </x:c>
-      <x:c r="G3" s="37" t="str">
         <x:v>CE 核對
 帶出</x:v>
       </x:c>
+      <x:c r="G3" s="37" t="str">
+        <x:v>CE 從來源帶出</x:v>
+      </x:c>
       <x:c r="H3" s="37" t="str">
-        <x:v>CE 從來源帶出</x:v>
+        <x:v>CE 從公司系統帶出</x:v>
       </x:c>
       <x:c r="I3" s="37" t="str">
-        <x:v>CE 從來源帶出</x:v>
+        <x:v>CE 從公司系統帶出</x:v>
       </x:c>
       <x:c r="J3" s="37" t="str">
-        <x:v>CE 從來源帶出</x:v>
+        <x:v>CE 查核後填寫</x:v>
       </x:c>
       <x:c r="K3" s="37" t="str">
-        <x:v>原始分組
-CE 保留</x:v>
+        <x:v>CE 從公司系統帶出</x:v>
       </x:c>
       <x:c r="L3" s="37" t="str">
-        <x:v>來源資料
-CE 保留</x:v>
-      </x:c>
-      <x:c r="M3" s="37" t="str">
-        <x:v>來源參考
-CE 保留</x:v>
-      </x:c>
-      <x:c r="N3" s="37" t="str">
-        <x:v>CE 從公司系統帶出</x:v>
-      </x:c>
-      <x:c r="O3" s="37" t="str">
-        <x:v>CE 查核後填寫</x:v>
-      </x:c>
-      <x:c r="P3" s="37" t="str">
-        <x:v>CE 從公司系統帶出</x:v>
-      </x:c>
-      <x:c r="Q3" s="37" t="str">
         <x:v>RD 原始
 CE 保留</x:v>
       </x:c>
-      <x:c r="R3" s="37" t="str">
+      <x:c r="M3" s="37" t="str">
         <x:v>原 BOM
 CE 保留</x:v>
       </x:c>
-      <x:c r="S3" s="37" t="str">
+      <x:c r="N3" s="37" t="str">
         <x:v>RD 原始
 CE 保留</x:v>
       </x:c>
-      <x:c r="T3" s="38" t="str">
+      <x:c r="O3" s="38" t="str">
         <x:v>CE 補欄
 帶出原文</x:v>
       </x:c>
@@ -1341,51 +1223,36 @@
         <x:v>Ref Des</x:v>
       </x:c>
       <x:c r="E4" s="19" t="str">
-        <x:v>Manufacturer Part Number(1)</x:v>
+        <x:v>Manufacturer Part Number</x:v>
       </x:c>
       <x:c r="F4" s="19" t="str">
-        <x:v>Manufacturer Part Number(2)</x:v>
+        <x:v>Manufacturer</x:v>
       </x:c>
       <x:c r="G4" s="19" t="str">
-        <x:v>Manufacturer</x:v>
+        <x:v>Sourcing Status</x:v>
       </x:c>
       <x:c r="H4" s="19" t="str">
-        <x:v>Sourcing Status</x:v>
+        <x:v>虛擬料號</x:v>
       </x:c>
       <x:c r="I4" s="19" t="str">
-        <x:v>Virtual PN</x:v>
+        <x:v>實體料號</x:v>
       </x:c>
       <x:c r="J4" s="19" t="str">
-        <x:v>PEGA P/N</x:v>
+        <x:v>Symbol</x:v>
       </x:c>
       <x:c r="K4" s="19" t="str">
-        <x:v>Ref_tmp</x:v>
+        <x:v>Part Name</x:v>
       </x:c>
       <x:c r="L4" s="19" t="str">
-        <x:v>LV</x:v>
+        <x:v>Part Spec</x:v>
       </x:c>
       <x:c r="M4" s="19" t="str">
-        <x:v>CIS/Remark</x:v>
+        <x:v>Schematic_Part</x:v>
       </x:c>
       <x:c r="N4" s="19" t="str">
-        <x:v>Part Number</x:v>
-      </x:c>
-      <x:c r="O4" s="19" t="str">
-        <x:v>Symbol</x:v>
-      </x:c>
-      <x:c r="P4" s="19" t="str">
-        <x:v>Part Name</x:v>
-      </x:c>
-      <x:c r="Q4" s="19" t="str">
-        <x:v>Part Spec</x:v>
-      </x:c>
-      <x:c r="R4" s="19" t="str">
-        <x:v>Schematic_Part</x:v>
-      </x:c>
-      <x:c r="S4" s="19" t="str">
         <x:v>PCB_Footprint</x:v>
       </x:c>
-      <x:c r="T4" s="20" t="str">
+      <x:c r="O4" s="20" t="str">
         <x:v>零件狀態</x:v>
       </x:c>
     </x:row>
@@ -1405,45 +1272,34 @@
       <x:c r="E5" s="45" t="str">
         <x:v>DEMO-CAP-001</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str"/>
+      <x:c r="F5" s="45" t="str">
+        <x:v>示範廠商 A</x:v>
+      </x:c>
       <x:c r="G5" s="45" t="str">
-        <x:v>示範廠商 A</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="H5" s="45" t="str">
-        <x:v>Approved</x:v>
+        <x:v>DEMO-VIRTUAL-001</x:v>
       </x:c>
       <x:c r="I5" s="45" t="str">
-        <x:v>DEMO-TX-001</x:v>
-      </x:c>
-      <x:c r="J5" s="45" t="str"/>
+        <x:v>000-DEMO-001</x:v>
+      </x:c>
+      <x:c r="J5" s="45" t="str">
+        <x:v>無</x:v>
+      </x:c>
       <x:c r="K5" s="45" t="str">
-        <x:v>C101, C102</x:v>
+        <x:v>示範電容</x:v>
       </x:c>
       <x:c r="L5" s="45" t="str">
-        <x:v>A</x:v>
+        <x:v>0.1uF / 16V / X7R</x:v>
       </x:c>
       <x:c r="M5" s="45" t="str">
-        <x:v>格式示範，非真實核准料</x:v>
+        <x:v>CAP</x:v>
       </x:c>
       <x:c r="N5" s="45" t="str">
-        <x:v>000-DEMO-001</x:v>
+        <x:v>C_0402</x:v>
       </x:c>
       <x:c r="O5" s="45" t="str">
-        <x:v>無</x:v>
-      </x:c>
-      <x:c r="P5" s="45" t="str">
-        <x:v>示範電容</x:v>
-      </x:c>
-      <x:c r="Q5" s="45" t="str">
-        <x:v>0.1uF / 16V / X7R</x:v>
-      </x:c>
-      <x:c r="R5" s="45" t="str">
-        <x:v>CAP</x:v>
-      </x:c>
-      <x:c r="S5" s="45" t="str">
-        <x:v>C_0402</x:v>
-      </x:c>
-      <x:c r="T5" s="45" t="str">
         <x:v>待確認</x:v>
       </x:c>
     </x:row>
@@ -1463,45 +1319,34 @@
       <x:c r="E6" s="46" t="str">
         <x:v>DEMO-CAP-ALT</x:v>
       </x:c>
-      <x:c r="F6" s="46" t="str"/>
+      <x:c r="F6" s="46" t="str">
+        <x:v>示範廠商 B</x:v>
+      </x:c>
       <x:c r="G6" s="46" t="str">
-        <x:v>示範廠商 B</x:v>
+        <x:v>Approved</x:v>
       </x:c>
       <x:c r="H6" s="46" t="str">
-        <x:v>Approved</x:v>
-      </x:c>
-      <x:c r="I6" s="46" t="str"/>
+        <x:v>DEMO-VIRTUAL-001</x:v>
+      </x:c>
+      <x:c r="I6" s="46" t="str">
+        <x:v>000-DEMO-ALT</x:v>
+      </x:c>
       <x:c r="J6" s="46" t="str">
-        <x:v>DEMO-PEGA-ALT</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="K6" s="46" t="str">
-        <x:v>C101, C102</x:v>
+        <x:v>示範替代電容</x:v>
       </x:c>
       <x:c r="L6" s="46" t="str">
-        <x:v>A</x:v>
+        <x:v>0.1uF / 16V / X7R</x:v>
       </x:c>
       <x:c r="M6" s="46" t="str">
-        <x:v>同位號候選料另列，RD 尚未確認</x:v>
+        <x:v>CAP</x:v>
       </x:c>
       <x:c r="N6" s="46" t="str">
-        <x:v>000-DEMO-ALT</x:v>
+        <x:v>C_0402</x:v>
       </x:c>
       <x:c r="O6" s="46" t="str">
-        <x:v>C</x:v>
-      </x:c>
-      <x:c r="P6" s="46" t="str">
-        <x:v>示範替代電容</x:v>
-      </x:c>
-      <x:c r="Q6" s="46" t="str">
-        <x:v>0.1uF / 16V / X7R</x:v>
-      </x:c>
-      <x:c r="R6" s="46" t="str">
-        <x:v>CAP</x:v>
-      </x:c>
-      <x:c r="S6" s="46" t="str">
-        <x:v>C_0402</x:v>
-      </x:c>
-      <x:c r="T6" s="46" t="str">
         <x:v>新設計產品不建議使用－ODM 不建議用料</x:v>
       </x:c>
     </x:row>
@@ -1521,43 +1366,34 @@
       <x:c r="E7" s="46" t="str">
         <x:v>DEMO-IC-EOL</x:v>
       </x:c>
-      <x:c r="F7" s="46" t="str"/>
+      <x:c r="F7" s="46" t="str">
+        <x:v>示範廠商 C</x:v>
+      </x:c>
       <x:c r="G7" s="46" t="str">
-        <x:v>示範廠商 C</x:v>
+        <x:v>Active</x:v>
       </x:c>
       <x:c r="H7" s="46" t="str">
-        <x:v>Active</x:v>
-      </x:c>
-      <x:c r="I7" s="46" t="str"/>
-      <x:c r="J7" s="46" t="str"/>
+        <x:v>DEMO-VIRTUAL-IC</x:v>
+      </x:c>
+      <x:c r="I7" s="46" t="str">
+        <x:v>000-DEMO-EOL</x:v>
+      </x:c>
+      <x:c r="J7" s="46" t="str">
+        <x:v>有</x:v>
+      </x:c>
       <x:c r="K7" s="46" t="str">
-        <x:v>U10</x:v>
+        <x:v>示範電源 IC</x:v>
       </x:c>
       <x:c r="L7" s="46" t="str">
-        <x:v>A</x:v>
+        <x:v>示範規格</x:v>
       </x:c>
       <x:c r="M7" s="46" t="str">
-        <x:v>Active 不代表新設計可用</x:v>
+        <x:v>POWER_IC</x:v>
       </x:c>
       <x:c r="N7" s="46" t="str">
-        <x:v>000-DEMO-EOL</x:v>
+        <x:v>QFN_DEMO</x:v>
       </x:c>
       <x:c r="O7" s="46" t="str">
-        <x:v>有</x:v>
-      </x:c>
-      <x:c r="P7" s="46" t="str">
-        <x:v>示範電源 IC</x:v>
-      </x:c>
-      <x:c r="Q7" s="46" t="str">
-        <x:v>示範規格</x:v>
-      </x:c>
-      <x:c r="R7" s="46" t="str">
-        <x:v>POWER_IC</x:v>
-      </x:c>
-      <x:c r="S7" s="46" t="str">
-        <x:v>QFN_DEMO</x:v>
-      </x:c>
-      <x:c r="T7" s="46" t="str">
         <x:v>新設計產品不建議使用－EOL</x:v>
       </x:c>
     </x:row>
@@ -1577,37 +1413,26 @@
       <x:c r="E8" s="47" t="str">
         <x:v>DEMO-CONN-NEW</x:v>
       </x:c>
-      <x:c r="F8" s="47" t="str"/>
-      <x:c r="G8" s="47" t="str">
+      <x:c r="F8" s="47" t="str">
         <x:v>示範廠商 D</x:v>
       </x:c>
+      <x:c r="G8" s="47" t="str"/>
       <x:c r="H8" s="47" t="str"/>
       <x:c r="I8" s="47" t="str"/>
-      <x:c r="J8" s="47" t="str"/>
-      <x:c r="K8" s="47" t="str">
-        <x:v>J20</x:v>
-      </x:c>
+      <x:c r="J8" s="47" t="str">
+        <x:v>無</x:v>
+      </x:c>
+      <x:c r="K8" s="47" t="str"/>
       <x:c r="L8" s="47" t="str">
-        <x:v>A</x:v>
+        <x:v>示範規格</x:v>
       </x:c>
       <x:c r="M8" s="47" t="str">
-        <x:v>查無公司料號；請 RD 確認後續處理</x:v>
-      </x:c>
-      <x:c r="N8" s="47" t="str"/>
+        <x:v>CONN</x:v>
+      </x:c>
+      <x:c r="N8" s="47" t="str">
+        <x:v>CONN_DEMO</x:v>
+      </x:c>
       <x:c r="O8" s="47" t="str">
-        <x:v>無</x:v>
-      </x:c>
-      <x:c r="P8" s="47" t="str"/>
-      <x:c r="Q8" s="47" t="str">
-        <x:v>示範規格</x:v>
-      </x:c>
-      <x:c r="R8" s="47" t="str">
-        <x:v>CONN</x:v>
-      </x:c>
-      <x:c r="S8" s="47" t="str">
-        <x:v>CONN_DEMO</x:v>
-      </x:c>
-      <x:c r="T8" s="47" t="str">
         <x:v>待確認</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
add CE field meanings and independent phase out and Symbol columns
</commit_message>
<xml_diff>
--- a/public/material-ce-reference.xlsx
+++ b/public/material-ce-reference.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分工與欄位說明" sheetId="1" r:id="R0c4ec5f9217b4f2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CE交付範例" sheetId="2" r:id="Ref6b92ebbffa442d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分工與欄位說明" sheetId="1" r:id="R2a555f952e264a19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CE交付範例" sheetId="2" r:id="R06bcce652c684b60"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +19,7 @@
     <x:numFmt numFmtId="201" formatCode="0"/>
     <x:numFmt numFmtId="202" formatCode="General"/>
   </x:numFmts>
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -57,8 +57,13 @@
       <x:color rgb="FF8B3E24"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF43566A"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -85,8 +90,13 @@
         <x:fgColor rgb="FFFFF0CC"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF0F6"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="8">
+  <x:borders count="11">
     <x:border>
       <x:left/>
       <x:right/>
@@ -161,11 +171,46 @@
       <x:bottom/>
       <x:diagonal/>
     </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFFFFFFF"/>
+      </x:right>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFCDD7E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFFFFFFF"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFFFFFFF"/>
+      </x:right>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFCDD7E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFFFFFFF"/>
+      </x:left>
+      <x:right/>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFCDD7E2"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="60">
+  <x:cellXfs count="71">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -275,6 +320,39 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -617,10 +695,10 @@
         <x:v>CE</x:v>
       </x:c>
       <x:c r="B7" s="22" t="str">
-        <x:v>整理後 BOM＋零件狀態</x:v>
+        <x:v>整理後 BOM＋各欄原值</x:v>
       </x:c>
       <x:c r="C7" s="22" t="str">
-        <x:v>依 RD 提供的客戶 BOM，利用公司現有系統整理並轉出清單；保留設計欄位，補上右側「零件狀態」，再交回 RD。查無料號或狀態不明時明確註記待確認。</x:v>
+        <x:v>依 RD 提供的 BOM 整理公司資料，保留設計欄位、虛實料號及各狀態欄原值，依格式填寫 phase out、Symbol 與零件狀態；未知處標示待確認。</x:v>
       </x:c>
       <x:c r="D7" s="3"/>
       <x:c r="E7" s="3"/>
@@ -646,7 +724,7 @@
         <x:v>確認結果與後續申請追蹤</x:v>
       </x:c>
       <x:c r="C9" s="22" t="str">
-        <x:v>提供設計 BOM，匯入 CE 清單後核對位號、用量、料號與零件狀態；依公司流程確認選用／申請事項，再於網站記錄追蹤說明、單號與更新人。</x:v>
+        <x:v>提供設計 BOM，匯入 CE 清單後逐欄核對；phase out、Symbol 各自獨立，不互相代填。依公司流程確認選用／申請事項，再於網站記錄追蹤說明、單號與更新人。</x:v>
       </x:c>
       <x:c r="D9" s="3"/>
       <x:c r="E9" s="3"/>
@@ -684,7 +762,7 @@
       </x:c>
       <x:c r="B13" s="23"/>
       <x:c r="C13" s="22" t="str">
-        <x:v>Sourcing Status 是供應／核准來源狀態；零件狀態是新設計使用限制。兩欄分開保留。Approved／Active 不代表可以忽略禁用或 ODM 不建議用料。</x:v>
+        <x:v>phase out 與 Symbol 是兩個獨立欄位。phase out 記錄零件狀態；Symbol 記錄是否已有實體料號但缺 Symbol。兩欄各自保留原值，不互相代填，也不改名或覆蓋其他欄位。</x:v>
       </x:c>
       <x:c r="D13" s="23"/>
       <x:c r="E13" s="23"/>
@@ -728,7 +806,7 @@
       </x:c>
       <x:c r="B17" s="23"/>
       <x:c r="C17" s="22" t="str">
-        <x:v>Symbol 填該實體料是否已建置 Symbol：有／無／待確認。已有實體料號、明確無 Symbol 時只補 Symbol；空白或 C 等未定義代碼保留原值，先待確認。Schematic_Part 另存符號名稱。</x:v>
+        <x:v>Symbol 的意思是是否已有實體料號但缺 Symbol；由 CE 依來源確認後填寫，網站獨立顯示原文。C 等未定義代碼照原值保留，不自行改填缺 Symbol 或已齊備。Schematic_Part 仍是符號名稱。</x:v>
       </x:c>
       <x:c r="D17" s="23"/>
       <x:c r="E17" s="23"/>
@@ -759,7 +837,7 @@
       </x:c>
       <x:c r="B20" s="23"/>
       <x:c r="C20" s="22" t="str">
-        <x:v>CE 利用公司現有系統核對並帶出虛擬料號、實體料號與供應狀態，在最右側補上零件狀態；未知處明確填待確認。</x:v>
+        <x:v>CE 利用公司現有系統帶出虛實料號及各欄原值，phase out 與 Symbol 分別填寫，不合併、不代填。</x:v>
       </x:c>
       <x:c r="D20" s="23"/>
       <x:c r="E20" s="23"/>
@@ -781,7 +859,7 @@
       </x:c>
       <x:c r="B22" s="23"/>
       <x:c r="C22" s="22" t="str">
-        <x:v>RD 使用上傳 BOM 匯入，核對位號、MPN、虛擬料號、實體料號、供應狀態與零件狀態。工具只整理與提示，不自動核准。</x:v>
+        <x:v>RD 使用上傳 BOM 匯入，逐欄核對位號、MPN、虛實料號、phase out、Symbol 與零件狀態。工具保留原值，不自動核准。</x:v>
       </x:c>
       <x:c r="D22" s="23"/>
       <x:c r="E22" s="23"/>
@@ -892,7 +970,7 @@
         <x:v>保留完整位號，逗號分隔；同組替代料使用相同位號。</x:v>
       </x:c>
       <x:c r="D30" s="28" t="str">
-        <x:v>REF DES</x:v>
+        <x:v>位號（REF DES）</x:v>
       </x:c>
       <x:c r="E30" s="32" t="str">
         <x:v>C101, C102</x:v>
@@ -909,7 +987,7 @@
         <x:v>每列只填一個廠商料號，搭配該列廠商及實體料號；同一虛擬料下的其他實體料另列。</x:v>
       </x:c>
       <x:c r="D31" s="28" t="str">
-        <x:v>MPN</x:v>
+        <x:v>廠商料號（MPN）</x:v>
       </x:c>
       <x:c r="E31" s="32" t="str">
         <x:v>DEMO-CAP-001</x:v>
@@ -940,7 +1018,7 @@
         <x:v>CE 從來源帶出</x:v>
       </x:c>
       <x:c r="C33" s="28" t="str">
-        <x:v>保留公司／原廠供應與核准狀態原文，例如 Approved、Active、NRND、Obsolete；不得用它取代右側零件狀態。</x:v>
+        <x:v>保留公司／原廠供應與核准狀態原文，例如 Approved；不得用它改填 phase out、Symbol 或最右側零件狀態。</x:v>
       </x:c>
       <x:c r="D33" s="28" t="str">
         <x:v>供應／核准狀態</x:v>
@@ -991,13 +1069,13 @@
         <x:v>CE 查核後填寫</x:v>
       </x:c>
       <x:c r="C36" s="28" t="str">
-        <x:v>填該實體料有沒有已建置 Symbol：有／無／待確認。已有實體料號且填無時只需補 Symbol；原始 C 等代碼保留，未定義前不判有無。</x:v>
+        <x:v>此欄獨立記錄是否已有實體料號但缺 Symbol，由 CE 依來源填寫；不因 phase out 或其他欄位而覆寫。C 等未定義代碼照原值保留，不自行轉成有、無或其他結論。</x:v>
       </x:c>
       <x:c r="D36" s="28" t="str">
-        <x:v>Symbol 建置狀態／缺件提示</x:v>
+        <x:v>Symbol（獨立原值）</x:v>
       </x:c>
       <x:c r="E36" s="32" t="str">
-        <x:v>有／無／待確認</x:v>
+        <x:v>來源原文；不明填待確認</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="34" customHeight="1">
@@ -1011,7 +1089,7 @@
         <x:v>來源有公司料名就保留；無資料可留白。</x:v>
       </x:c>
       <x:c r="D37" s="28" t="str">
-        <x:v>內部料名</x:v>
+        <x:v>實體料名</x:v>
       </x:c>
       <x:c r="E37" s="32" t="str">
         <x:v>示範電容</x:v>
@@ -1028,7 +1106,7 @@
         <x:v>保留原規格；同組資料維持一致，差異交 RD 確認。</x:v>
       </x:c>
       <x:c r="D38" s="28" t="str">
-        <x:v>規格</x:v>
+        <x:v>料件規格</x:v>
       </x:c>
       <x:c r="E38" s="32" t="str">
         <x:v>0.1uF / 16V / X7R</x:v>
@@ -1062,26 +1140,43 @@
         <x:v>原 BOM 有封裝就保留；無資料可留白，不要求 CE 新建封裝。</x:v>
       </x:c>
       <x:c r="D40" s="28" t="str">
-        <x:v>Footprint</x:v>
+        <x:v>PCB 封裝名稱</x:v>
       </x:c>
       <x:c r="E40" s="32" t="str">
         <x:v>C_0402</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="34" customHeight="1">
-      <x:c r="A41" s="29" t="str">
+      <x:c r="A41" s="27" t="str">
+        <x:v>phase out</x:v>
+      </x:c>
+      <x:c r="B41" s="27" t="str">
+        <x:v>CE 從公司系統帶出</x:v>
+      </x:c>
+      <x:c r="C41" s="28" t="str">
+        <x:v>此欄獨立保留公司的零件狀態原文，例如 ACTIVE、PHASEOUT、UNDERREVIEW；不與 Symbol 合併，也不覆寫其他狀態欄。</x:v>
+      </x:c>
+      <x:c r="D41" s="28" t="str">
+        <x:v>phase out（獨立原值）</x:v>
+      </x:c>
+      <x:c r="E41" s="32" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42" ht="34" customHeight="1">
+      <x:c r="A42" s="29" t="str">
         <x:v>零件狀態</x:v>
       </x:c>
-      <x:c r="B41" s="29" t="str">
+      <x:c r="B42" s="29" t="str">
         <x:v>CE 補欄／帶出原文</x:v>
       </x:c>
-      <x:c r="C41" s="30" t="str">
-        <x:v>本次交付必須補在最右側。填公司新設計使用限制原文；不明填待確認，供 RD 後續確認與參考。</x:v>
-      </x:c>
-      <x:c r="D41" s="30" t="str">
-        <x:v>零件狀態（獨立顯示）</x:v>
-      </x:c>
-      <x:c r="E41" s="33" t="str">
+      <x:c r="C42" s="30" t="str">
+        <x:v>本次交付保留在最右側，填公司來源原文，例如 ODM 不建議用料；不明填待確認。此既有欄位不因新增 phase out 或 Symbol 而改名或改值。</x:v>
+      </x:c>
+      <x:c r="D42" s="30" t="str">
+        <x:v>零件狀態（原欄位）</x:v>
+      </x:c>
+      <x:c r="E42" s="33" t="str">
         <x:v>新設計產品不建議使用－ODM 不建議用料</x:v>
       </x:c>
     </x:row>
@@ -1106,12 +1201,13 @@
     <x:col min="7" max="7" width="25" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="25" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="28" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="26" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="28" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="25" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="30" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="25" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="25" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="45" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="30" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="45" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1132,10 +1228,11 @@
       <x:c r="M1" s="6"/>
       <x:c r="N1" s="6"/>
       <x:c r="O1" s="6"/>
+      <x:c r="P1" s="6"/>
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="34" t="str">
-        <x:v>範例中的料號、廠商與狀態都是格式示範，不能當成真實選料、核准或替代料相容性依據。</x:v>
+        <x:v>第4列表頭、第5列中文說明請保留，第6列起為 DEMO 範例。範例中的料號、廠商與狀態都是格式示範，不能當成真實選料、核准或替代料相容性依據。</x:v>
       </x:c>
       <x:c r="B2" s="3"/>
       <x:c r="C2" s="3"/>
@@ -1151,6 +1248,7 @@
       <x:c r="M2" s="3"/>
       <x:c r="N2" s="3"/>
       <x:c r="O2" s="3"/>
+      <x:c r="P2" s="3"/>
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="37" t="str">
@@ -1204,7 +1302,10 @@
         <x:v>RD 原始
 CE 保留</x:v>
       </x:c>
-      <x:c r="O3" s="38" t="str">
+      <x:c r="O3" s="37" t="str">
+        <x:v>CE 從公司系統帶出</x:v>
+      </x:c>
+      <x:c r="P3" s="38" t="str">
         <x:v>CE 補欄
 帶出原文</x:v>
       </x:c>
@@ -1252,187 +1353,252 @@
       <x:c r="N4" s="19" t="str">
         <x:v>PCB_Footprint</x:v>
       </x:c>
-      <x:c r="O4" s="20" t="str">
+      <x:c r="O4" s="19" t="str">
+        <x:v>phase out</x:v>
+      </x:c>
+      <x:c r="P4" s="20" t="str">
         <x:v>零件狀態</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="42" customHeight="1">
-      <x:c r="A5" s="54" t="n">
+    <x:row r="5" ht="52" customHeight="1">
+      <x:c r="A5" s="47" t="str">
+        <x:v>階層：0 系統／1 模組／2 料件</x:v>
+      </x:c>
+      <x:c r="B5" s="48" t="str">
+        <x:v>設計 BOM 的料件名稱</x:v>
+      </x:c>
+      <x:c r="C5" s="48" t="str">
+        <x:v>單一產品的用量</x:v>
+      </x:c>
+      <x:c r="D5" s="48" t="str">
+        <x:v>電路位號，例如 C101、R1</x:v>
+      </x:c>
+      <x:c r="E5" s="48" t="str">
+        <x:v>單一廠商的單一原廠料號（MPN）</x:v>
+      </x:c>
+      <x:c r="F5" s="48" t="str">
+        <x:v>該列 MPN 的製造商</x:v>
+      </x:c>
+      <x:c r="G5" s="48" t="str">
+        <x:v>供應／核准來源狀態，保留原文</x:v>
+      </x:c>
+      <x:c r="H5" s="48" t="str">
+        <x:v>可共用多個實體料的上層料號</x:v>
+      </x:c>
+      <x:c r="I5" s="48" t="str">
+        <x:v>已申請的單一廠商、單一 MPN 實體料號</x:v>
+      </x:c>
+      <x:c r="J5" s="48" t="str">
+        <x:v>是否已有實體料號但缺 Symbol（保留原文）</x:v>
+      </x:c>
+      <x:c r="K5" s="48" t="str">
+        <x:v>實體料號對應的公司料名</x:v>
+      </x:c>
+      <x:c r="L5" s="48" t="str">
+        <x:v>料件規格，保留原內容</x:v>
+      </x:c>
+      <x:c r="M5" s="48" t="str">
+        <x:v>原理圖符號名稱，不代表 Symbol 有無</x:v>
+      </x:c>
+      <x:c r="N5" s="48" t="str">
+        <x:v>PCB 封裝名稱</x:v>
+      </x:c>
+      <x:c r="O5" s="48" t="str">
+        <x:v>零件狀態（保留公司原文）</x:v>
+      </x:c>
+      <x:c r="P5" s="49" t="str">
+        <x:v>新設計使用限制；不明填待確認</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="42" customHeight="1">
+      <x:c r="A6" s="65" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B5" s="45" t="str">
+      <x:c r="B6" s="56" t="str">
         <x:v>CAP CER 0.1UF 16V X7R</x:v>
       </x:c>
-      <x:c r="C5" s="57" t="n">
+      <x:c r="C6" s="68" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D5" s="45" t="str">
+      <x:c r="D6" s="56" t="str">
         <x:v>C101, C102</x:v>
       </x:c>
-      <x:c r="E5" s="45" t="str">
+      <x:c r="E6" s="56" t="str">
         <x:v>DEMO-CAP-001</x:v>
       </x:c>
-      <x:c r="F5" s="45" t="str">
+      <x:c r="F6" s="56" t="str">
         <x:v>示範廠商 A</x:v>
       </x:c>
-      <x:c r="G5" s="45" t="str">
+      <x:c r="G6" s="56" t="str">
         <x:v>Approved</x:v>
       </x:c>
-      <x:c r="H5" s="45" t="str">
+      <x:c r="H6" s="56" t="str">
         <x:v>DEMO-VIRTUAL-001</x:v>
       </x:c>
-      <x:c r="I5" s="45" t="str">
+      <x:c r="I6" s="56" t="str">
         <x:v>000-DEMO-001</x:v>
       </x:c>
-      <x:c r="J5" s="45" t="str">
+      <x:c r="J6" s="56" t="str">
         <x:v>無</x:v>
       </x:c>
-      <x:c r="K5" s="45" t="str">
+      <x:c r="K6" s="56" t="str">
         <x:v>示範電容</x:v>
       </x:c>
-      <x:c r="L5" s="45" t="str">
+      <x:c r="L6" s="56" t="str">
         <x:v>0.1uF / 16V / X7R</x:v>
       </x:c>
-      <x:c r="M5" s="45" t="str">
+      <x:c r="M6" s="56" t="str">
         <x:v>CAP</x:v>
       </x:c>
-      <x:c r="N5" s="45" t="str">
+      <x:c r="N6" s="56" t="str">
         <x:v>C_0402</x:v>
       </x:c>
-      <x:c r="O5" s="45" t="str">
+      <x:c r="O6" s="56" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="P6" s="56" t="str">
         <x:v>待確認</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="42" customHeight="1">
-      <x:c r="A6" s="55" t="n">
+    <x:row r="7" ht="42" customHeight="1">
+      <x:c r="A7" s="66" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B6" s="46" t="str">
+      <x:c r="B7" s="57" t="str">
         <x:v>CAP CER 0.1UF 16V X7R</x:v>
       </x:c>
-      <x:c r="C6" s="58" t="n">
+      <x:c r="C7" s="69" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="D6" s="46" t="str">
+      <x:c r="D7" s="57" t="str">
         <x:v>C101, C102</x:v>
       </x:c>
-      <x:c r="E6" s="46" t="str">
+      <x:c r="E7" s="57" t="str">
         <x:v>DEMO-CAP-ALT</x:v>
       </x:c>
-      <x:c r="F6" s="46" t="str">
+      <x:c r="F7" s="57" t="str">
         <x:v>示範廠商 B</x:v>
       </x:c>
-      <x:c r="G6" s="46" t="str">
+      <x:c r="G7" s="57" t="str">
         <x:v>Approved</x:v>
       </x:c>
-      <x:c r="H6" s="46" t="str">
+      <x:c r="H7" s="57" t="str">
         <x:v>DEMO-VIRTUAL-001</x:v>
       </x:c>
-      <x:c r="I6" s="46" t="str">
+      <x:c r="I7" s="57" t="str">
         <x:v>000-DEMO-ALT</x:v>
       </x:c>
-      <x:c r="J6" s="46" t="str">
+      <x:c r="J7" s="57" t="str">
         <x:v>C</x:v>
       </x:c>
-      <x:c r="K6" s="46" t="str">
+      <x:c r="K7" s="57" t="str">
         <x:v>示範替代電容</x:v>
       </x:c>
-      <x:c r="L6" s="46" t="str">
+      <x:c r="L7" s="57" t="str">
         <x:v>0.1uF / 16V / X7R</x:v>
       </x:c>
-      <x:c r="M6" s="46" t="str">
+      <x:c r="M7" s="57" t="str">
         <x:v>CAP</x:v>
       </x:c>
-      <x:c r="N6" s="46" t="str">
+      <x:c r="N7" s="57" t="str">
         <x:v>C_0402</x:v>
       </x:c>
-      <x:c r="O6" s="46" t="str">
+      <x:c r="O7" s="57" t="str">
+        <x:v>ACTIVE</x:v>
+      </x:c>
+      <x:c r="P7" s="57" t="str">
         <x:v>新設計產品不建議使用－ODM 不建議用料</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="42" customHeight="1">
-      <x:c r="A7" s="55" t="n">
+    <x:row r="8" ht="42" customHeight="1">
+      <x:c r="A8" s="66" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B7" s="46" t="str">
+      <x:c r="B8" s="57" t="str">
         <x:v>POWER IC</x:v>
       </x:c>
-      <x:c r="C7" s="58" t="n">
+      <x:c r="C8" s="69" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D7" s="46" t="str">
+      <x:c r="D8" s="57" t="str">
         <x:v>U10</x:v>
       </x:c>
-      <x:c r="E7" s="46" t="str">
+      <x:c r="E8" s="57" t="str">
         <x:v>DEMO-IC-EOL</x:v>
       </x:c>
-      <x:c r="F7" s="46" t="str">
+      <x:c r="F8" s="57" t="str">
         <x:v>示範廠商 C</x:v>
       </x:c>
-      <x:c r="G7" s="46" t="str">
+      <x:c r="G8" s="57" t="str">
         <x:v>Active</x:v>
       </x:c>
-      <x:c r="H7" s="46" t="str">
+      <x:c r="H8" s="57" t="str">
         <x:v>DEMO-VIRTUAL-IC</x:v>
       </x:c>
-      <x:c r="I7" s="46" t="str">
+      <x:c r="I8" s="57" t="str">
         <x:v>000-DEMO-EOL</x:v>
       </x:c>
-      <x:c r="J7" s="46" t="str">
+      <x:c r="J8" s="57" t="str">
         <x:v>有</x:v>
       </x:c>
-      <x:c r="K7" s="46" t="str">
+      <x:c r="K8" s="57" t="str">
         <x:v>示範電源 IC</x:v>
       </x:c>
-      <x:c r="L7" s="46" t="str">
+      <x:c r="L8" s="57" t="str">
         <x:v>示範規格</x:v>
       </x:c>
-      <x:c r="M7" s="46" t="str">
+      <x:c r="M8" s="57" t="str">
         <x:v>POWER_IC</x:v>
       </x:c>
-      <x:c r="N7" s="46" t="str">
+      <x:c r="N8" s="57" t="str">
         <x:v>QFN_DEMO</x:v>
       </x:c>
-      <x:c r="O7" s="46" t="str">
+      <x:c r="O8" s="57" t="str">
+        <x:v>PHASEOUT</x:v>
+      </x:c>
+      <x:c r="P8" s="57" t="str">
         <x:v>新設計產品不建議使用－EOL</x:v>
       </x:c>
     </x:row>
-    <x:row r="8" ht="42" customHeight="1">
-      <x:c r="A8" s="56" t="n">
+    <x:row r="9" ht="42" customHeight="1">
+      <x:c r="A9" s="67" t="n">
         <x:v>2</x:v>
       </x:c>
-      <x:c r="B8" s="47" t="str">
+      <x:c r="B9" s="58" t="str">
         <x:v>CONNECTOR</x:v>
       </x:c>
-      <x:c r="C8" s="59" t="n">
+      <x:c r="C9" s="70" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="D8" s="47" t="str">
+      <x:c r="D9" s="58" t="str">
         <x:v>J20</x:v>
       </x:c>
-      <x:c r="E8" s="47" t="str">
+      <x:c r="E9" s="58" t="str">
         <x:v>DEMO-CONN-NEW</x:v>
       </x:c>
-      <x:c r="F8" s="47" t="str">
+      <x:c r="F9" s="58" t="str">
         <x:v>示範廠商 D</x:v>
       </x:c>
-      <x:c r="G8" s="47" t="str"/>
-      <x:c r="H8" s="47" t="str"/>
-      <x:c r="I8" s="47" t="str"/>
-      <x:c r="J8" s="47" t="str">
+      <x:c r="G9" s="58" t="str"/>
+      <x:c r="H9" s="58" t="str"/>
+      <x:c r="I9" s="58" t="str"/>
+      <x:c r="J9" s="58" t="str">
         <x:v>無</x:v>
       </x:c>
-      <x:c r="K8" s="47" t="str"/>
-      <x:c r="L8" s="47" t="str">
+      <x:c r="K9" s="58" t="str"/>
+      <x:c r="L9" s="58" t="str">
         <x:v>示範規格</x:v>
       </x:c>
-      <x:c r="M8" s="47" t="str">
+      <x:c r="M9" s="58" t="str">
         <x:v>CONN</x:v>
       </x:c>
-      <x:c r="N8" s="47" t="str">
+      <x:c r="N9" s="58" t="str">
         <x:v>CONN_DEMO</x:v>
       </x:c>
-      <x:c r="O8" s="47" t="str">
+      <x:c r="O9" s="58" t="str">
+        <x:v>UNDERREVIEW</x:v>
+      </x:c>
+      <x:c r="P9" s="58" t="str">
         <x:v>待確認</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
adopt user CE format and remove standalone Symbol
</commit_message>
<xml_diff>
--- a/public/material-ce-reference.xlsx
+++ b/public/material-ce-reference.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分工與欄位說明" sheetId="1" r:id="R2a555f952e264a19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CE交付範例" sheetId="2" r:id="R06bcce652c684b60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="分工與欄位說明" sheetId="1" r:id="R2d67d2e10974401d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CE交付範例" sheetId="2" r:id="R184494dbe4c740f8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -698,7 +698,7 @@
         <x:v>整理後 BOM＋各欄原值</x:v>
       </x:c>
       <x:c r="C7" s="22" t="str">
-        <x:v>依 RD 提供的 BOM 整理公司資料，保留設計欄位、虛實料號及各狀態欄原值，依格式填寫 phase out、Symbol 與零件狀態；未知處標示待確認。</x:v>
+        <x:v>依 RD 提供的 BOM 整理公司資料，保留虛實料號及狀態原值；依交付格式核對原理圖符號，確認 OrCAD 能叫出該符號，再交回 RD。</x:v>
       </x:c>
       <x:c r="D7" s="3"/>
       <x:c r="E7" s="3"/>
@@ -724,7 +724,7 @@
         <x:v>確認結果與後續申請追蹤</x:v>
       </x:c>
       <x:c r="C9" s="22" t="str">
-        <x:v>提供設計 BOM，匯入 CE 清單後逐欄核對；phase out、Symbol 各自獨立，不互相代填。依公司流程確認選用／申請事項，再於網站記錄追蹤說明、單號與更新人。</x:v>
+        <x:v>提供設計 BOM，匯入 CE 清單後逐欄核對；依公司流程確認選用／申請事項，再於網站記錄追蹤說明、單號與更新人。</x:v>
       </x:c>
       <x:c r="D9" s="3"/>
       <x:c r="E9" s="3"/>
@@ -762,7 +762,7 @@
       </x:c>
       <x:c r="B13" s="23"/>
       <x:c r="C13" s="22" t="str">
-        <x:v>phase out 與 Symbol 是兩個獨立欄位。phase out 記錄零件狀態；Symbol 記錄是否已有實體料號但缺 Symbol。兩欄各自保留原值，不互相代填，也不改名或覆蓋其他欄位。</x:v>
+        <x:v>依使用者提供的交付檔保留 15 欄，不再另填 Symbol 欄。Schematic_Part 記錄供 OrCAD 叫出的原理圖符號；phase out 與零件狀態各自保留原文。</x:v>
       </x:c>
       <x:c r="D13" s="23"/>
       <x:c r="E13" s="23"/>
@@ -806,7 +806,7 @@
       </x:c>
       <x:c r="B17" s="23"/>
       <x:c r="C17" s="22" t="str">
-        <x:v>Symbol 的意思是是否已有實體料號但缺 Symbol；由 CE 依來源確認後填寫，網站獨立顯示原文。C 等未定義代碼照原值保留，不自行改填缺 Symbol 或已齊備。Schematic_Part 仍是符號名稱。</x:v>
+        <x:v>Schematic_Part：原理圖符號(orcad要能叫出原理圖符號)。由 CE 在 OrCAD 核對後填寫；網站保留欄位內容，不因填有文字就宣稱已驗證可叫出，也不額外推算 Symbol 缺件。</x:v>
       </x:c>
       <x:c r="D17" s="23"/>
       <x:c r="E17" s="23"/>
@@ -837,7 +837,7 @@
       </x:c>
       <x:c r="B20" s="23"/>
       <x:c r="C20" s="22" t="str">
-        <x:v>CE 利用公司現有系統帶出虛實料號及各欄原值，phase out 與 Symbol 分別填寫，不合併、不代填。</x:v>
+        <x:v>CE 利用公司現有系統帶出虛實料號及各欄原值，並核對 Schematic_Part 的原理圖符號可由 OrCAD 叫出。</x:v>
       </x:c>
       <x:c r="D20" s="23"/>
       <x:c r="E20" s="23"/>
@@ -859,7 +859,7 @@
       </x:c>
       <x:c r="B22" s="23"/>
       <x:c r="C22" s="22" t="str">
-        <x:v>RD 使用上傳 BOM 匯入，逐欄核對位號、MPN、虛實料號、phase out、Symbol 與零件狀態。工具保留原值，不自動核准。</x:v>
+        <x:v>RD 使用上傳 BOM 匯入，逐欄核對位號、MPN、虛實料號、Schematic_Part、phase out 與零件狀態。工具保留原值，不自動核准。</x:v>
       </x:c>
       <x:c r="D22" s="23"/>
       <x:c r="E22" s="23"/>
@@ -1018,7 +1018,7 @@
         <x:v>CE 從來源帶出</x:v>
       </x:c>
       <x:c r="C33" s="28" t="str">
-        <x:v>保留公司／原廠供應與核准狀態原文，例如 Approved；不得用它改填 phase out、Symbol 或最右側零件狀態。</x:v>
+        <x:v>保留公司／原廠供應與核准狀態原文，例如 Approved；不得用它改填 phase out 或最右側零件狀態。</x:v>
       </x:c>
       <x:c r="D33" s="28" t="str">
         <x:v>供應／核准狀態</x:v>
@@ -1061,122 +1061,105 @@
         <x:v>000-DEMO-001</x:v>
       </x:c>
     </x:row>
-    <x:row r="36" ht="52" customHeight="1">
+    <x:row r="36" ht="34" customHeight="1">
       <x:c r="A36" s="27" t="str">
-        <x:v>Symbol</x:v>
+        <x:v>Part Name</x:v>
       </x:c>
       <x:c r="B36" s="27" t="str">
-        <x:v>CE 查核後填寫</x:v>
+        <x:v>CE 從公司系統帶出</x:v>
       </x:c>
       <x:c r="C36" s="28" t="str">
-        <x:v>此欄獨立記錄是否已有實體料號但缺 Symbol，由 CE 依來源填寫；不因 phase out 或其他欄位而覆寫。C 等未定義代碼照原值保留，不自行轉成有、無或其他結論。</x:v>
+        <x:v>來源有公司料名就保留；無資料可留白。</x:v>
       </x:c>
       <x:c r="D36" s="28" t="str">
-        <x:v>Symbol（獨立原值）</x:v>
+        <x:v>實體料名</x:v>
       </x:c>
       <x:c r="E36" s="32" t="str">
-        <x:v>來源原文；不明填待確認</x:v>
+        <x:v>示範電容</x:v>
       </x:c>
     </x:row>
     <x:row r="37" ht="34" customHeight="1">
       <x:c r="A37" s="27" t="str">
-        <x:v>Part Name</x:v>
+        <x:v>Part Spec</x:v>
       </x:c>
       <x:c r="B37" s="27" t="str">
-        <x:v>CE 從公司系統帶出</x:v>
+        <x:v>RD 原始／CE 保留</x:v>
       </x:c>
       <x:c r="C37" s="28" t="str">
-        <x:v>來源有公司料名就保留；無資料可留白。</x:v>
+        <x:v>保留原規格；同組資料維持一致，差異交 RD 確認。</x:v>
       </x:c>
       <x:c r="D37" s="28" t="str">
-        <x:v>實體料名</x:v>
+        <x:v>料件規格</x:v>
       </x:c>
       <x:c r="E37" s="32" t="str">
-        <x:v>示範電容</x:v>
+        <x:v>0.1uF / 16V / X7R</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="34" customHeight="1">
       <x:c r="A38" s="27" t="str">
-        <x:v>Part Spec</x:v>
+        <x:v>Schematic_Part</x:v>
       </x:c>
       <x:c r="B38" s="27" t="str">
-        <x:v>RD 原始／CE 保留</x:v>
+        <x:v>CE 核對／帶出</x:v>
       </x:c>
       <x:c r="C38" s="28" t="str">
-        <x:v>保留原規格；同組資料維持一致，差異交 RD 確認。</x:v>
+        <x:v>填寫 OrCAD 能叫出的原理圖符號，依來源核對後保留內容；不另填 Symbol 有無或缺件欄。網站不會將文字存在視為已完成 OrCAD 驗證。</x:v>
       </x:c>
       <x:c r="D38" s="28" t="str">
-        <x:v>料件規格</x:v>
+        <x:v>原理圖符號（Schematic_Part）</x:v>
       </x:c>
       <x:c r="E38" s="32" t="str">
-        <x:v>0.1uF / 16V / X7R</x:v>
+        <x:v>CAP</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="34" customHeight="1">
       <x:c r="A39" s="27" t="str">
-        <x:v>Schematic_Part</x:v>
+        <x:v>PCB_Footprint</x:v>
       </x:c>
       <x:c r="B39" s="27" t="str">
-        <x:v>原 BOM／CE 保留</x:v>
+        <x:v>RD 原始／CE 保留</x:v>
       </x:c>
       <x:c r="C39" s="28" t="str">
-        <x:v>原 BOM 的符號名稱，例如 CAP；這欄不代表 Symbol 是否已建置，有無狀態請填 Symbol 欄。</x:v>
+        <x:v>保留零件 footprint 的來源內容；無資料可留白，不要求 CE 為填表另建封裝。</x:v>
       </x:c>
       <x:c r="D39" s="28" t="str">
-        <x:v>原理圖符號名稱</x:v>
+        <x:v>零件 footprint</x:v>
       </x:c>
       <x:c r="E39" s="32" t="str">
-        <x:v>CAP</x:v>
+        <x:v>C_0402</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="34" customHeight="1">
       <x:c r="A40" s="27" t="str">
-        <x:v>PCB_Footprint</x:v>
+        <x:v>phase out</x:v>
       </x:c>
       <x:c r="B40" s="27" t="str">
-        <x:v>RD 原始／CE 保留</x:v>
+        <x:v>CE 從公司系統帶出</x:v>
       </x:c>
       <x:c r="C40" s="28" t="str">
-        <x:v>原 BOM 有封裝就保留；無資料可留白，不要求 CE 新建封裝。</x:v>
+        <x:v>此欄獨立保留公司的零件狀態原文，例如 ACTIVE、PHASEOUT、UNDERREVIEW，不覆寫其他狀態欄。</x:v>
       </x:c>
       <x:c r="D40" s="28" t="str">
-        <x:v>PCB 封裝名稱</x:v>
+        <x:v>phase out（獨立原值）</x:v>
       </x:c>
       <x:c r="E40" s="32" t="str">
-        <x:v>C_0402</x:v>
+        <x:v>ACTIVE</x:v>
       </x:c>
     </x:row>
     <x:row r="41" ht="34" customHeight="1">
-      <x:c r="A41" s="27" t="str">
-        <x:v>phase out</x:v>
-      </x:c>
-      <x:c r="B41" s="27" t="str">
-        <x:v>CE 從公司系統帶出</x:v>
-      </x:c>
-      <x:c r="C41" s="28" t="str">
-        <x:v>此欄獨立保留公司的零件狀態原文，例如 ACTIVE、PHASEOUT、UNDERREVIEW；不與 Symbol 合併，也不覆寫其他狀態欄。</x:v>
-      </x:c>
-      <x:c r="D41" s="28" t="str">
-        <x:v>phase out（獨立原值）</x:v>
-      </x:c>
-      <x:c r="E41" s="32" t="str">
-        <x:v>ACTIVE</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="42" ht="34" customHeight="1">
-      <x:c r="A42" s="29" t="str">
+      <x:c r="A41" s="29" t="str">
         <x:v>零件狀態</x:v>
       </x:c>
-      <x:c r="B42" s="29" t="str">
+      <x:c r="B41" s="29" t="str">
         <x:v>CE 補欄／帶出原文</x:v>
       </x:c>
-      <x:c r="C42" s="30" t="str">
-        <x:v>本次交付保留在最右側，填公司來源原文，例如 ODM 不建議用料；不明填待確認。此既有欄位不因新增 phase out 或 Symbol 而改名或改值。</x:v>
-      </x:c>
-      <x:c r="D42" s="30" t="str">
+      <x:c r="C41" s="30" t="str">
+        <x:v>保留最右側欄位與公司來源原文，例如 ODM 不建議用料；不明填待確認，不改名或改值。</x:v>
+      </x:c>
+      <x:c r="D41" s="30" t="str">
         <x:v>零件狀態（原欄位）</x:v>
       </x:c>
-      <x:c r="E42" s="33" t="str">
+      <x:c r="E41" s="33" t="str">
         <x:v>新設計產品不建議使用－ODM 不建議用料</x:v>
       </x:c>
     </x:row>
@@ -1201,13 +1184,12 @@
     <x:col min="7" max="7" width="25" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="25" hidden="0" customWidth="1"/>
     <x:col min="9" max="9" width="28" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="28" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="25" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="30" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="25" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="30" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="25" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="25" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="25" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="30" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="45" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="30" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="45" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1228,7 +1210,6 @@
       <x:c r="M1" s="6"/>
       <x:c r="N1" s="6"/>
       <x:c r="O1" s="6"/>
-      <x:c r="P1" s="6"/>
     </x:row>
     <x:row r="2" ht="27" customHeight="1">
       <x:c r="A2" s="34" t="str">
@@ -1248,7 +1229,6 @@
       <x:c r="M2" s="3"/>
       <x:c r="N2" s="3"/>
       <x:c r="O2" s="3"/>
-      <x:c r="P2" s="3"/>
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
       <x:c r="A3" s="37" t="str">
@@ -1285,27 +1265,24 @@
         <x:v>CE 從公司系統帶出</x:v>
       </x:c>
       <x:c r="J3" s="37" t="str">
-        <x:v>CE 查核後填寫</x:v>
+        <x:v>CE 從公司系統帶出</x:v>
       </x:c>
       <x:c r="K3" s="37" t="str">
-        <x:v>CE 從公司系統帶出</x:v>
-      </x:c>
-      <x:c r="L3" s="37" t="str">
         <x:v>RD 原始
 CE 保留</x:v>
       </x:c>
+      <x:c r="L3" s="37" t="str">
+        <x:v>CE 核對
+帶出</x:v>
+      </x:c>
       <x:c r="M3" s="37" t="str">
-        <x:v>原 BOM
-CE 保留</x:v>
-      </x:c>
-      <x:c r="N3" s="37" t="str">
         <x:v>RD 原始
 CE 保留</x:v>
       </x:c>
-      <x:c r="O3" s="37" t="str">
+      <x:c r="N3" s="37" t="str">
         <x:v>CE 從公司系統帶出</x:v>
       </x:c>
-      <x:c r="P3" s="38" t="str">
+      <x:c r="O3" s="38" t="str">
         <x:v>CE 補欄
 帶出原文</x:v>
       </x:c>
@@ -1339,24 +1316,21 @@
         <x:v>實體料號</x:v>
       </x:c>
       <x:c r="J4" s="19" t="str">
-        <x:v>Symbol</x:v>
+        <x:v>Part Name</x:v>
       </x:c>
       <x:c r="K4" s="19" t="str">
-        <x:v>Part Name</x:v>
+        <x:v>Part Spec</x:v>
       </x:c>
       <x:c r="L4" s="19" t="str">
-        <x:v>Part Spec</x:v>
+        <x:v>Schematic_Part</x:v>
       </x:c>
       <x:c r="M4" s="19" t="str">
-        <x:v>Schematic_Part</x:v>
+        <x:v>PCB_Footprint</x:v>
       </x:c>
       <x:c r="N4" s="19" t="str">
-        <x:v>PCB_Footprint</x:v>
-      </x:c>
-      <x:c r="O4" s="19" t="str">
         <x:v>phase out</x:v>
       </x:c>
-      <x:c r="P4" s="20" t="str">
+      <x:c r="O4" s="20" t="str">
         <x:v>零件狀態</x:v>
       </x:c>
     </x:row>
@@ -1389,24 +1363,21 @@
         <x:v>已申請的單一廠商、單一 MPN 實體料號</x:v>
       </x:c>
       <x:c r="J5" s="48" t="str">
-        <x:v>是否已有實體料號但缺 Symbol（保留原文）</x:v>
+        <x:v>實體料號對應的公司料名</x:v>
       </x:c>
       <x:c r="K5" s="48" t="str">
-        <x:v>實體料號對應的公司料名</x:v>
+        <x:v>料件規格，保留原內容</x:v>
       </x:c>
       <x:c r="L5" s="48" t="str">
-        <x:v>料件規格，保留原內容</x:v>
+        <x:v>原理圖符號(orcad要能叫出原理圖符號)</x:v>
       </x:c>
       <x:c r="M5" s="48" t="str">
-        <x:v>原理圖符號名稱，不代表 Symbol 有無</x:v>
+        <x:v>零件footprint</x:v>
       </x:c>
       <x:c r="N5" s="48" t="str">
-        <x:v>PCB 封裝名稱</x:v>
-      </x:c>
-      <x:c r="O5" s="48" t="str">
         <x:v>零件狀態（保留公司原文）</x:v>
       </x:c>
-      <x:c r="P5" s="49" t="str">
+      <x:c r="O5" s="49" t="str">
         <x:v>新設計使用限制；不明填待確認</x:v>
       </x:c>
     </x:row>
@@ -1439,24 +1410,21 @@
         <x:v>000-DEMO-001</x:v>
       </x:c>
       <x:c r="J6" s="56" t="str">
-        <x:v>無</x:v>
+        <x:v>示範電容</x:v>
       </x:c>
       <x:c r="K6" s="56" t="str">
-        <x:v>示範電容</x:v>
+        <x:v>0.1uF / 16V / X7R</x:v>
       </x:c>
       <x:c r="L6" s="56" t="str">
-        <x:v>0.1uF / 16V / X7R</x:v>
+        <x:v>CAP</x:v>
       </x:c>
       <x:c r="M6" s="56" t="str">
-        <x:v>CAP</x:v>
+        <x:v>C_0402</x:v>
       </x:c>
       <x:c r="N6" s="56" t="str">
-        <x:v>C_0402</x:v>
+        <x:v>ACTIVE</x:v>
       </x:c>
       <x:c r="O6" s="56" t="str">
-        <x:v>ACTIVE</x:v>
-      </x:c>
-      <x:c r="P6" s="56" t="str">
         <x:v>待確認</x:v>
       </x:c>
     </x:row>
@@ -1489,24 +1457,21 @@
         <x:v>000-DEMO-ALT</x:v>
       </x:c>
       <x:c r="J7" s="57" t="str">
-        <x:v>C</x:v>
+        <x:v>示範替代電容</x:v>
       </x:c>
       <x:c r="K7" s="57" t="str">
-        <x:v>示範替代電容</x:v>
+        <x:v>0.1uF / 16V / X7R</x:v>
       </x:c>
       <x:c r="L7" s="57" t="str">
-        <x:v>0.1uF / 16V / X7R</x:v>
+        <x:v>CAP</x:v>
       </x:c>
       <x:c r="M7" s="57" t="str">
-        <x:v>CAP</x:v>
+        <x:v>C_0402</x:v>
       </x:c>
       <x:c r="N7" s="57" t="str">
-        <x:v>C_0402</x:v>
+        <x:v>ACTIVE</x:v>
       </x:c>
       <x:c r="O7" s="57" t="str">
-        <x:v>ACTIVE</x:v>
-      </x:c>
-      <x:c r="P7" s="57" t="str">
         <x:v>新設計產品不建議使用－ODM 不建議用料</x:v>
       </x:c>
     </x:row>
@@ -1539,24 +1504,21 @@
         <x:v>000-DEMO-EOL</x:v>
       </x:c>
       <x:c r="J8" s="57" t="str">
-        <x:v>有</x:v>
+        <x:v>示範電源 IC</x:v>
       </x:c>
       <x:c r="K8" s="57" t="str">
-        <x:v>示範電源 IC</x:v>
+        <x:v>示範規格</x:v>
       </x:c>
       <x:c r="L8" s="57" t="str">
-        <x:v>示範規格</x:v>
+        <x:v>POWER_IC</x:v>
       </x:c>
       <x:c r="M8" s="57" t="str">
-        <x:v>POWER_IC</x:v>
+        <x:v>QFN_DEMO</x:v>
       </x:c>
       <x:c r="N8" s="57" t="str">
-        <x:v>QFN_DEMO</x:v>
+        <x:v>PHASEOUT</x:v>
       </x:c>
       <x:c r="O8" s="57" t="str">
-        <x:v>PHASEOUT</x:v>
-      </x:c>
-      <x:c r="P8" s="57" t="str">
         <x:v>新設計產品不建議使用－EOL</x:v>
       </x:c>
     </x:row>
@@ -1582,23 +1544,20 @@
       <x:c r="G9" s="58" t="str"/>
       <x:c r="H9" s="58" t="str"/>
       <x:c r="I9" s="58" t="str"/>
-      <x:c r="J9" s="58" t="str">
-        <x:v>無</x:v>
-      </x:c>
-      <x:c r="K9" s="58" t="str"/>
+      <x:c r="J9" s="58" t="str"/>
+      <x:c r="K9" s="58" t="str">
+        <x:v>示範規格</x:v>
+      </x:c>
       <x:c r="L9" s="58" t="str">
-        <x:v>示範規格</x:v>
+        <x:v>CONN</x:v>
       </x:c>
       <x:c r="M9" s="58" t="str">
-        <x:v>CONN</x:v>
+        <x:v>CONN_DEMO</x:v>
       </x:c>
       <x:c r="N9" s="58" t="str">
-        <x:v>CONN_DEMO</x:v>
+        <x:v>UNDERREVIEW</x:v>
       </x:c>
       <x:c r="O9" s="58" t="str">
-        <x:v>UNDERREVIEW</x:v>
-      </x:c>
-      <x:c r="P9" s="58" t="str">
         <x:v>待確認</x:v>
       </x:c>
     </x:row>

</xml_diff>